<commit_message>
Pooh Points: normal 20260304
</commit_message>
<xml_diff>
--- a/docs/Today_PoohPoints_SEC_ByOwner_2026-03-04.xlsx
+++ b/docs/Today_PoohPoints_SEC_ByOwner_2026-03-04.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V151"/>
+  <dimension ref="A1:V152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -429,7 +429,7 @@
     <col width="26" customWidth="1" min="4" max="4"/>
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
     <col width="6" customWidth="1" min="8" max="8"/>
     <col width="5" customWidth="1" min="9" max="9"/>
     <col width="5" customWidth="1" min="10" max="10"/>
@@ -1233,12 +1233,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Billy Richmond III</t>
+          <t>Matas Vokietaitis</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1248,53 +1248,53 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="I10" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="J10" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P10" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="Q10" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="R10" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="S10" t="n">
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U10" t="n">
         <v>2</v>
       </c>
       <c r="V10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="11">
@@ -1315,12 +1315,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Matas Vokietaitis</t>
+          <t>Billy Richmond III</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1330,53 +1330,53 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H11" t="n">
+        <v>12</v>
+      </c>
+      <c r="I11" t="n">
+        <v>4</v>
+      </c>
+      <c r="J11" t="n">
         <v>6</v>
       </c>
-      <c r="I11" t="n">
-        <v>10</v>
-      </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2</v>
+      </c>
+      <c r="M11" t="n">
+        <v>3</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" t="n">
         <v>5</v>
       </c>
-      <c r="K11" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
-      </c>
-      <c r="M11" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" t="n">
-        <v>1</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="n">
-        <v>13</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>4</v>
-      </c>
-      <c r="R11" t="n">
-        <v>10</v>
-      </c>
       <c r="S11" t="n">
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U11" t="n">
         <v>2</v>
       </c>
       <c r="V11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="12">
@@ -1412,14 +1412,14 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H12" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I12" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J12" t="n">
         <v>1</v>
@@ -1440,7 +1440,7 @@
         <v>2</v>
       </c>
       <c r="P12" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="Q12" t="n">
         <v>2</v>
@@ -1455,10 +1455,10 @@
         <v>1</v>
       </c>
       <c r="U12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="V12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
@@ -2232,23 +2232,23 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H22" t="n">
+        <v>24</v>
+      </c>
+      <c r="I22" t="n">
         <v>17</v>
       </c>
-      <c r="I22" t="n">
-        <v>11</v>
-      </c>
       <c r="J22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M22" t="n">
         <v>3</v>
@@ -2260,25 +2260,25 @@
         <v>0</v>
       </c>
       <c r="P22" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="Q22" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="R22" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="S22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -2327,10 +2327,10 @@
         <v>2</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M23" t="n">
         <v>1</v>
@@ -2339,22 +2339,22 @@
         <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="P23" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="Q23" t="n">
         <v>3</v>
       </c>
       <c r="R23" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="S23" t="n">
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U23" t="n">
         <v>4</v>
@@ -4118,14 +4118,14 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J45" t="n">
         <v>1</v>
@@ -4146,7 +4146,7 @@
         <v>3</v>
       </c>
       <c r="P45" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="Q45" t="n">
         <v>1</v>
@@ -4161,10 +4161,10 @@
         <v>0</v>
       </c>
       <c r="U45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -4938,53 +4938,53 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H55" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="I55" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="J55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K55" t="n">
+        <v>8</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0</v>
+      </c>
+      <c r="N55" t="n">
+        <v>2</v>
+      </c>
+      <c r="O55" t="n">
+        <v>1</v>
+      </c>
+      <c r="P55" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q55" t="n">
         <v>6</v>
       </c>
-      <c r="L55" t="n">
-        <v>0</v>
-      </c>
-      <c r="M55" t="n">
-        <v>0</v>
-      </c>
-      <c r="N55" t="n">
-        <v>1</v>
-      </c>
-      <c r="O55" t="n">
-        <v>1</v>
-      </c>
-      <c r="P55" t="n">
-        <v>15</v>
-      </c>
-      <c r="Q55" t="n">
-        <v>2</v>
-      </c>
       <c r="R55" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="S55" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T55" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="U55" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V55" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56">
@@ -5020,7 +5020,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H56" t="n">
@@ -5045,7 +5045,7 @@
         <v>0</v>
       </c>
       <c r="O56" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="P56" t="n">
         <v>4</v>
@@ -5840,7 +5840,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H66" t="n">
@@ -5850,10 +5850,10 @@
         <v>10</v>
       </c>
       <c r="J66" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L66" t="n">
         <v>0</v>
@@ -5862,19 +5862,19 @@
         <v>1</v>
       </c>
       <c r="N66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O66" t="n">
         <v>0</v>
       </c>
       <c r="P66" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="Q66" t="n">
         <v>3</v>
       </c>
       <c r="R66" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="S66" t="n">
         <v>0</v>
@@ -12400,7 +12400,7 @@
       </c>
       <c r="G146" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H146" t="n">
@@ -12410,7 +12410,7 @@
         <v>3</v>
       </c>
       <c r="J146" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K146" t="n">
         <v>0</v>
@@ -12422,13 +12422,13 @@
         <v>0</v>
       </c>
       <c r="N146" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O146" t="n">
         <v>0</v>
       </c>
       <c r="P146" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="Q146" t="n">
         <v>1</v>
@@ -12482,11 +12482,11 @@
       </c>
       <c r="G147" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H147" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I147" t="n">
         <v>2</v>
@@ -12510,13 +12510,13 @@
         <v>1</v>
       </c>
       <c r="P147" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="Q147" t="n">
         <v>1</v>
       </c>
       <c r="R147" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S147" t="n">
         <v>0</v>
@@ -12564,7 +12564,7 @@
       </c>
       <c r="G148" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H148" t="n">
@@ -12646,11 +12646,11 @@
       </c>
       <c r="G149" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H149" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I149" t="n">
         <v>2</v>
@@ -12674,13 +12674,13 @@
         <v>1</v>
       </c>
       <c r="P149" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="Q149" t="n">
         <v>1</v>
       </c>
       <c r="R149" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="S149" t="n">
         <v>0</v>
@@ -12728,7 +12728,7 @@
       </c>
       <c r="G150" t="inlineStr">
         <is>
-          <t>2:46 - 1st Half</t>
+          <t>19:51 - 2nd Half</t>
         </is>
       </c>
       <c r="H150" t="n">
@@ -12738,7 +12738,7 @@
         <v>0</v>
       </c>
       <c r="J150" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K150" t="n">
         <v>1</v>
@@ -12756,19 +12756,19 @@
         <v>1</v>
       </c>
       <c r="P150" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="Q150" t="n">
         <v>0</v>
       </c>
       <c r="R150" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S150" t="n">
         <v>0</v>
       </c>
       <c r="T150" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="U150" t="n">
         <v>0</v>
@@ -12795,67 +12795,149 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
+          <t>Isaiah Sealy</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>ARK</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>TEX@ARK</t>
+        </is>
+      </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>19:51 - 2nd Half</t>
+        </is>
+      </c>
+      <c r="H151" t="n">
+        <v>0</v>
+      </c>
+      <c r="I151" t="n">
+        <v>0</v>
+      </c>
+      <c r="J151" t="n">
+        <v>0</v>
+      </c>
+      <c r="K151" t="n">
+        <v>0</v>
+      </c>
+      <c r="L151" t="n">
+        <v>0</v>
+      </c>
+      <c r="M151" t="n">
+        <v>0</v>
+      </c>
+      <c r="N151" t="n">
+        <v>0</v>
+      </c>
+      <c r="O151" t="n">
+        <v>0</v>
+      </c>
+      <c r="P151" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q151" t="n">
+        <v>0</v>
+      </c>
+      <c r="R151" t="n">
+        <v>0</v>
+      </c>
+      <c r="S151" t="n">
+        <v>0</v>
+      </c>
+      <c r="T151" t="n">
+        <v>0</v>
+      </c>
+      <c r="U151" t="n">
+        <v>0</v>
+      </c>
+      <c r="V151" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Undrafted</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D152" t="inlineStr">
+        <is>
           <t>Simeon Wilcher</t>
         </is>
       </c>
-      <c r="E151" t="inlineStr">
+      <c r="E152" t="inlineStr">
         <is>
           <t>TEX</t>
         </is>
       </c>
-      <c r="F151" t="inlineStr">
+      <c r="F152" t="inlineStr">
         <is>
           <t>TEX@ARK</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>2:46 - 1st Half</t>
-        </is>
-      </c>
-      <c r="H151" t="n">
-        <v>-2</v>
-      </c>
-      <c r="I151" t="n">
-        <v>0</v>
-      </c>
-      <c r="J151" t="n">
-        <v>0</v>
-      </c>
-      <c r="K151" t="n">
-        <v>0</v>
-      </c>
-      <c r="L151" t="n">
-        <v>0</v>
-      </c>
-      <c r="M151" t="n">
-        <v>0</v>
-      </c>
-      <c r="N151" t="n">
-        <v>0</v>
-      </c>
-      <c r="O151" t="n">
-        <v>0</v>
-      </c>
-      <c r="P151" t="n">
-        <v>10</v>
-      </c>
-      <c r="Q151" t="n">
-        <v>0</v>
-      </c>
-      <c r="R151" t="n">
-        <v>1</v>
-      </c>
-      <c r="S151" t="n">
-        <v>0</v>
-      </c>
-      <c r="T151" t="n">
-        <v>0</v>
-      </c>
-      <c r="U151" t="n">
-        <v>0</v>
-      </c>
-      <c r="V151" t="n">
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>19:51 - 2nd Half</t>
+        </is>
+      </c>
+      <c r="H152" t="n">
+        <v>-3</v>
+      </c>
+      <c r="I152" t="n">
+        <v>0</v>
+      </c>
+      <c r="J152" t="n">
+        <v>0</v>
+      </c>
+      <c r="K152" t="n">
+        <v>1</v>
+      </c>
+      <c r="L152" t="n">
+        <v>0</v>
+      </c>
+      <c r="M152" t="n">
+        <v>0</v>
+      </c>
+      <c r="N152" t="n">
+        <v>1</v>
+      </c>
+      <c r="O152" t="n">
+        <v>0</v>
+      </c>
+      <c r="P152" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q152" t="n">
+        <v>0</v>
+      </c>
+      <c r="R152" t="n">
+        <v>2</v>
+      </c>
+      <c r="S152" t="n">
+        <v>0</v>
+      </c>
+      <c r="T152" t="n">
+        <v>1</v>
+      </c>
+      <c r="U152" t="n">
+        <v>0</v>
+      </c>
+      <c r="V152" t="n">
         <v>1</v>
       </c>
     </row>
@@ -12937,24 +13019,24 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Hilton Heads</t>
+          <t>The Backslashers</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>The Backslashers</t>
+          <t>Boozers Losers</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="C6" t="n">
         <v>4</v>
@@ -12963,14 +13045,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Boozers Losers</t>
+          <t>Hilton Heads</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>52</v>
+        <v>62</v>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -12980,7 +13062,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="C8" t="n">
         <v>5</v>

</xml_diff>

<commit_message>
Pooh Points: final 20260304 -> PD18
</commit_message>
<xml_diff>
--- a/docs/Today_PoohPoints_SEC_ByOwner_2026-03-04.xlsx
+++ b/docs/Today_PoohPoints_SEC_ByOwner_2026-03-04.xlsx
@@ -12795,12 +12795,12 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Declan Duru Jr.</t>
+          <t>Isaiah Sealy</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>TEX</t>
+          <t>ARK</t>
         </is>
       </c>
       <c r="F151" t="inlineStr">
@@ -12814,13 +12814,13 @@
         </is>
       </c>
       <c r="H151" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I151" t="n">
         <v>0</v>
       </c>
       <c r="J151" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K151" t="n">
         <v>0</v>
@@ -12835,10 +12835,10 @@
         <v>0</v>
       </c>
       <c r="O151" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P151" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q151" t="n">
         <v>0</v>
@@ -12877,12 +12877,12 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Isaiah Sealy</t>
+          <t>Declan Duru Jr.</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>ARK</t>
+          <t>TEX</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -12920,7 +12920,7 @@
         <v>0</v>
       </c>
       <c r="P152" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q152" t="n">
         <v>0</v>

</xml_diff>